<commit_message>
Make rooms feel live: 70+ online and unlabeled names
Keep community presence on the server so every room shows at least 70 people online, drifting slowly. Chat shows member names only—no AI/bot tags—and replies read like group-chat messages instead of a labeled simulation.

Co-authored-by: cjmatheka <cjmatheka@gmail.com>
</commit_message>
<xml_diff>
--- a/seed/personas.xlsx
+++ b/seed/personas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H86"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,13 +442,13 @@
         <v>curious</v>
       </c>
       <c r="F2" t="str">
-        <v>questions-first</v>
+        <v>casual</v>
       </c>
       <c r="G2" t="str">
         <v>general</v>
       </c>
       <c r="H2" t="str">
-        <v>moderate</v>
+        <v>low</v>
       </c>
     </row>
     <row r="3">
@@ -456,13 +456,13 @@
         <v>P-1002</v>
       </c>
       <c r="B3" t="str">
-        <v>Omar Voss</v>
+        <v>Omar Hock</v>
       </c>
       <c r="C3" t="str">
         <v>Toronto</v>
       </c>
       <c r="D3" t="str">
-        <v>experienced</v>
+        <v>intermediate</v>
       </c>
       <c r="E3" t="str">
         <v>practical</v>
@@ -474,7 +474,7 @@
         <v>procedural</v>
       </c>
       <c r="H3" t="str">
-        <v>high</v>
+        <v>moderate</v>
       </c>
     </row>
     <row r="4">
@@ -482,25 +482,25 @@
         <v>P-1003</v>
       </c>
       <c r="B4" t="str">
-        <v>Sable Wren</v>
+        <v>Sable Diallo</v>
       </c>
       <c r="C4" t="str">
         <v>Nairobi</v>
       </c>
       <c r="D4" t="str">
-        <v>intermediate</v>
+        <v>experienced</v>
       </c>
       <c r="E4" t="str">
         <v>analytical</v>
       </c>
       <c r="F4" t="str">
-        <v>compare-and-cite</v>
+        <v>conversational</v>
       </c>
       <c r="G4" t="str">
-        <v>docs-first</v>
+        <v>community</v>
       </c>
       <c r="H4" t="str">
-        <v>moderate</v>
+        <v>high</v>
       </c>
     </row>
     <row r="5">
@@ -508,13 +508,13 @@
         <v>P-1004</v>
       </c>
       <c r="B5" t="str">
-        <v>Jun Park</v>
+        <v>Jun Novak</v>
       </c>
       <c r="C5" t="str">
         <v>Seoul</v>
       </c>
       <c r="D5" t="str">
-        <v>experienced</v>
+        <v>beginner</v>
       </c>
       <c r="E5" t="str">
         <v>calm</v>
@@ -523,7 +523,7 @@
         <v>plain-language</v>
       </c>
       <c r="G5" t="str">
-        <v>policy</v>
+        <v>onboarding</v>
       </c>
       <c r="H5" t="str">
         <v>low</v>
@@ -534,13 +534,13 @@
         <v>P-1005</v>
       </c>
       <c r="B6" t="str">
-        <v>Mira Solis</v>
+        <v>Mira Okafor</v>
       </c>
       <c r="C6" t="str">
         <v>Mexico City</v>
       </c>
       <c r="D6" t="str">
-        <v>beginner</v>
+        <v>intermediate</v>
       </c>
       <c r="E6" t="str">
         <v>enthusiastic</v>
@@ -549,10 +549,10 @@
         <v>warm</v>
       </c>
       <c r="G6" t="str">
-        <v>overview</v>
+        <v>faq</v>
       </c>
       <c r="H6" t="str">
-        <v>high</v>
+        <v>moderate</v>
       </c>
     </row>
     <row r="7">
@@ -560,13 +560,13 @@
         <v>P-1006</v>
       </c>
       <c r="B7" t="str">
-        <v>Theo Brandt</v>
+        <v>Theo Jensen</v>
       </c>
       <c r="C7" t="str">
         <v>Berlin</v>
       </c>
       <c r="D7" t="str">
-        <v>intermediate</v>
+        <v>experienced</v>
       </c>
       <c r="E7" t="str">
         <v>skeptical</v>
@@ -575,10 +575,10 @@
         <v>precise</v>
       </c>
       <c r="G7" t="str">
-        <v>constraints</v>
+        <v>general</v>
       </c>
       <c r="H7" t="str">
-        <v>low</v>
+        <v>high</v>
       </c>
     </row>
     <row r="8">
@@ -586,25 +586,25 @@
         <v>P-1007</v>
       </c>
       <c r="B8" t="str">
-        <v>Asha Reddy</v>
+        <v>Asha Wren</v>
       </c>
       <c r="C8" t="str">
         <v>Hyderabad</v>
       </c>
       <c r="D8" t="str">
-        <v>experienced</v>
+        <v>beginner</v>
       </c>
       <c r="E8" t="str">
-        <v>practical</v>
+        <v>supportive</v>
       </c>
       <c r="F8" t="str">
-        <v>stepwise</v>
+        <v>casual</v>
       </c>
       <c r="G8" t="str">
-        <v>procedures</v>
+        <v>procedural</v>
       </c>
       <c r="H8" t="str">
-        <v>moderate</v>
+        <v>low</v>
       </c>
     </row>
     <row r="9">
@@ -612,22 +612,22 @@
         <v>P-1008</v>
       </c>
       <c r="B9" t="str">
-        <v>Lina Höck</v>
+        <v>Lina Rossi</v>
       </c>
       <c r="C9" t="str">
         <v>Vienna</v>
       </c>
       <c r="D9" t="str">
-        <v>beginner</v>
+        <v>intermediate</v>
       </c>
       <c r="E9" t="str">
-        <v>curious</v>
+        <v>reserved</v>
       </c>
       <c r="F9" t="str">
-        <v>casual</v>
+        <v>concise</v>
       </c>
       <c r="G9" t="str">
-        <v>faq</v>
+        <v>community</v>
       </c>
       <c r="H9" t="str">
         <v>moderate</v>
@@ -638,16 +638,16 @@
         <v>P-1009</v>
       </c>
       <c r="B10" t="str">
-        <v>Chris Adeyemi</v>
+        <v>Chris Khan</v>
       </c>
       <c r="C10" t="str">
         <v>Lagos</v>
       </c>
       <c r="D10" t="str">
-        <v>intermediate</v>
+        <v>experienced</v>
       </c>
       <c r="E10" t="str">
-        <v>supportive</v>
+        <v>playful</v>
       </c>
       <c r="F10" t="str">
         <v>conversational</v>
@@ -664,22 +664,22 @@
         <v>P-1010</v>
       </c>
       <c r="B11" t="str">
-        <v>Elena Rossi</v>
+        <v>Elena Moreau</v>
       </c>
       <c r="C11" t="str">
         <v>Milan</v>
       </c>
       <c r="D11" t="str">
-        <v>experienced</v>
+        <v>beginner</v>
       </c>
       <c r="E11" t="str">
-        <v>analytical</v>
+        <v>curious</v>
       </c>
       <c r="F11" t="str">
-        <v>structured</v>
+        <v>plain-language</v>
       </c>
       <c r="G11" t="str">
-        <v>terminology</v>
+        <v>faq</v>
       </c>
       <c r="H11" t="str">
         <v>low</v>
@@ -690,22 +690,22 @@
         <v>P-1011</v>
       </c>
       <c r="B12" t="str">
-        <v>Quinn Hale</v>
+        <v>Quinn Santos</v>
       </c>
       <c r="C12" t="str">
         <v>Austin</v>
       </c>
       <c r="D12" t="str">
-        <v>beginner</v>
+        <v>intermediate</v>
       </c>
       <c r="E12" t="str">
-        <v>playful</v>
+        <v>practical</v>
       </c>
       <c r="F12" t="str">
-        <v>short-messages</v>
+        <v>warm</v>
       </c>
       <c r="G12" t="str">
-        <v>community</v>
+        <v>general</v>
       </c>
       <c r="H12" t="str">
         <v>moderate</v>
@@ -716,7 +716,7 @@
         <v>P-1012</v>
       </c>
       <c r="B13" t="str">
-        <v>Priya Menon</v>
+        <v>Priya Kaur</v>
       </c>
       <c r="C13" t="str">
         <v>Singapore</v>
@@ -725,21 +725,1919 @@
         <v>experienced</v>
       </c>
       <c r="E13" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F13" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G13" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H13" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>P-1013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Mateo Solis</v>
+      </c>
+      <c r="C14" t="str">
+        <v>São Paulo</v>
+      </c>
+      <c r="D14" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E14" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F14" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G14" t="str">
+        <v>community</v>
+      </c>
+      <c r="H14" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>P-1014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Hana Menon</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Osaka</v>
+      </c>
+      <c r="D15" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E15" t="str">
+        <v>enthusiastic</v>
+      </c>
+      <c r="F15" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G15" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H15" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>P-1015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Ibrahim Nilsen</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Cairo</v>
+      </c>
+      <c r="D16" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E16" t="str">
+        <v>skeptical</v>
+      </c>
+      <c r="F16" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G16" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H16" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>P-1016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Sofia Costa</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Stockholm</v>
+      </c>
+      <c r="D17" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E17" t="str">
+        <v>supportive</v>
+      </c>
+      <c r="F17" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G17" t="str">
+        <v>general</v>
+      </c>
+      <c r="H17" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>P-1017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Leo Farouk</v>
+      </c>
+      <c r="C18" t="str">
+        <v>London</v>
+      </c>
+      <c r="D18" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E18" t="str">
         <v>reserved</v>
       </c>
-      <c r="F13" t="str">
-        <v>careful</v>
-      </c>
-      <c r="G13" t="str">
-        <v>safety</v>
-      </c>
-      <c r="H13" t="str">
+      <c r="F18" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G18" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H18" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>P-1018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Amara Frost</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Accra</v>
+      </c>
+      <c r="D19" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E19" t="str">
+        <v>playful</v>
+      </c>
+      <c r="F19" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G19" t="str">
+        <v>community</v>
+      </c>
+      <c r="H19" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>P-1019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Diego Reddy</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Chicago</v>
+      </c>
+      <c r="D20" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E20" t="str">
+        <v>curious</v>
+      </c>
+      <c r="F20" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G20" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H20" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>P-1020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Yara Okada</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="D21" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E21" t="str">
+        <v>practical</v>
+      </c>
+      <c r="F21" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G21" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H21" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>P-1021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Noah Silva</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Lisbon</v>
+      </c>
+      <c r="D22" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E22" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F22" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G22" t="str">
+        <v>general</v>
+      </c>
+      <c r="H22" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>P-1022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Leila Keller</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Toronto</v>
+      </c>
+      <c r="D23" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E23" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F23" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G23" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H23" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>P-1023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Kenji Petrov</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Nairobi</v>
+      </c>
+      <c r="D24" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E24" t="str">
+        <v>enthusiastic</v>
+      </c>
+      <c r="F24" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G24" t="str">
+        <v>community</v>
+      </c>
+      <c r="H24" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>P-1024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Freya Voss</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Seoul</v>
+      </c>
+      <c r="D25" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E25" t="str">
+        <v>skeptical</v>
+      </c>
+      <c r="F25" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G25" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H25" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>P-1025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Ravi Adeyemi</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Mexico City</v>
+      </c>
+      <c r="D26" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E26" t="str">
+        <v>supportive</v>
+      </c>
+      <c r="F26" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G26" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H26" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>P-1026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Ines Berg</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Berlin</v>
+      </c>
+      <c r="D27" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E27" t="str">
+        <v>reserved</v>
+      </c>
+      <c r="F27" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G27" t="str">
+        <v>general</v>
+      </c>
+      <c r="H27" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>P-1027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Malik Ibrahim</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="D28" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E28" t="str">
+        <v>playful</v>
+      </c>
+      <c r="F28" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G28" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H28" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>P-1028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Clara Lind</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Vienna</v>
+      </c>
+      <c r="D29" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E29" t="str">
+        <v>curious</v>
+      </c>
+      <c r="F29" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G29" t="str">
+        <v>community</v>
+      </c>
+      <c r="H29" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>P-1029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Hassan Mwangi</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Lagos</v>
+      </c>
+      <c r="D30" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E30" t="str">
+        <v>practical</v>
+      </c>
+      <c r="F30" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G30" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H30" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>P-1030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>June Park</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Milan</v>
+      </c>
+      <c r="D31" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E31" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F31" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G31" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H31" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>P-1031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Andre Hale</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Austin</v>
+      </c>
+      <c r="D32" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E32" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F32" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G32" t="str">
+        <v>general</v>
+      </c>
+      <c r="H32" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>P-1032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Noor Duarte</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Singapore</v>
+      </c>
+      <c r="D33" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E33" t="str">
+        <v>enthusiastic</v>
+      </c>
+      <c r="F33" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G33" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H33" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>P-1033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Felix Patel</v>
+      </c>
+      <c r="C34" t="str">
+        <v>São Paulo</v>
+      </c>
+      <c r="D34" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E34" t="str">
+        <v>skeptical</v>
+      </c>
+      <c r="F34" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G34" t="str">
+        <v>community</v>
+      </c>
+      <c r="H34" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>P-1034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Zara Bauer</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Osaka</v>
+      </c>
+      <c r="D35" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E35" t="str">
+        <v>supportive</v>
+      </c>
+      <c r="F35" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G35" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H35" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>P-1035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Hugo Romano</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Cairo</v>
+      </c>
+      <c r="D36" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E36" t="str">
+        <v>reserved</v>
+      </c>
+      <c r="F36" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G36" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H36" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>P-1036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Mei Brandt</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Stockholm</v>
+      </c>
+      <c r="D37" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E37" t="str">
+        <v>playful</v>
+      </c>
+      <c r="F37" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G37" t="str">
+        <v>general</v>
+      </c>
+      <c r="H37" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>P-1037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Samir Alvarez</v>
+      </c>
+      <c r="C38" t="str">
+        <v>London</v>
+      </c>
+      <c r="D38" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E38" t="str">
+        <v>curious</v>
+      </c>
+      <c r="F38" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G38" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H38" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>P-1038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Iris Cho</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Accra</v>
+      </c>
+      <c r="D39" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E39" t="str">
+        <v>practical</v>
+      </c>
+      <c r="F39" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G39" t="str">
+        <v>community</v>
+      </c>
+      <c r="H39" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>P-1039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Pavel Rahman</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Chicago</v>
+      </c>
+      <c r="D40" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E40" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F40" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G40" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H40" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>P-1040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Amina Nguyen</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="D41" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E41" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F41" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G41" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H41" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>P-1041</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Jonah Calder</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Lisbon</v>
+      </c>
+      <c r="D42" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E42" t="str">
+        <v>enthusiastic</v>
+      </c>
+      <c r="F42" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G42" t="str">
+        <v>general</v>
+      </c>
+      <c r="H42" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>P-1042</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Lucia Hock</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Toronto</v>
+      </c>
+      <c r="D43" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E43" t="str">
+        <v>skeptical</v>
+      </c>
+      <c r="F43" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G43" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H43" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>P-1043</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Tariq Diallo</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Nairobi</v>
+      </c>
+      <c r="D44" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E44" t="str">
+        <v>supportive</v>
+      </c>
+      <c r="F44" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G44" t="str">
+        <v>community</v>
+      </c>
+      <c r="H44" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>P-1044</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Eva Novak</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Seoul</v>
+      </c>
+      <c r="D45" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E45" t="str">
+        <v>reserved</v>
+      </c>
+      <c r="F45" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G45" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H45" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>P-1045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Nico Okafor</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Mexico City</v>
+      </c>
+      <c r="D46" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E46" t="str">
+        <v>playful</v>
+      </c>
+      <c r="F46" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G46" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H46" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>P-1046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Sana Jensen</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Berlin</v>
+      </c>
+      <c r="D47" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E47" t="str">
+        <v>curious</v>
+      </c>
+      <c r="F47" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G47" t="str">
+        <v>general</v>
+      </c>
+      <c r="H47" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>P-1047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Owen Wren</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="D48" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E48" t="str">
+        <v>practical</v>
+      </c>
+      <c r="F48" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G48" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H48" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>P-1048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Dalia Rossi</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Vienna</v>
+      </c>
+      <c r="D49" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E49" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F49" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G49" t="str">
+        <v>community</v>
+      </c>
+      <c r="H49" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>P-1049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Marco Khan</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Lagos</v>
+      </c>
+      <c r="D50" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E50" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F50" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G50" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H50" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>P-1050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Keiko Moreau</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Milan</v>
+      </c>
+      <c r="D51" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E51" t="str">
+        <v>enthusiastic</v>
+      </c>
+      <c r="F51" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G51" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H51" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>P-1051</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Adrian Santos</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Austin</v>
+      </c>
+      <c r="D52" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E52" t="str">
+        <v>skeptical</v>
+      </c>
+      <c r="F52" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G52" t="str">
+        <v>general</v>
+      </c>
+      <c r="H52" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>P-1052</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Nora Kaur</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Singapore</v>
+      </c>
+      <c r="D53" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E53" t="str">
+        <v>supportive</v>
+      </c>
+      <c r="F53" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G53" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H53" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>P-1053</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Yusuf Solis</v>
+      </c>
+      <c r="C54" t="str">
+        <v>São Paulo</v>
+      </c>
+      <c r="D54" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E54" t="str">
+        <v>reserved</v>
+      </c>
+      <c r="F54" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G54" t="str">
+        <v>community</v>
+      </c>
+      <c r="H54" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>P-1054</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Greta Menon</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Osaka</v>
+      </c>
+      <c r="D55" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E55" t="str">
+        <v>playful</v>
+      </c>
+      <c r="F55" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G55" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H55" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>P-1055</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Ilan Nilsen</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Cairo</v>
+      </c>
+      <c r="D56" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E56" t="str">
+        <v>curious</v>
+      </c>
+      <c r="F56" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G56" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H56" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>P-1056</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Rosa Costa</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Stockholm</v>
+      </c>
+      <c r="D57" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E57" t="str">
+        <v>practical</v>
+      </c>
+      <c r="F57" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G57" t="str">
+        <v>general</v>
+      </c>
+      <c r="H57" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>P-1057</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Kofi Farouk</v>
+      </c>
+      <c r="C58" t="str">
+        <v>London</v>
+      </c>
+      <c r="D58" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E58" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F58" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G58" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H58" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>P-1058</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Anika Frost</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Accra</v>
+      </c>
+      <c r="D59" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E59" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F59" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G59" t="str">
+        <v>community</v>
+      </c>
+      <c r="H59" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>P-1059</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Seth Reddy</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Chicago</v>
+      </c>
+      <c r="D60" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E60" t="str">
+        <v>enthusiastic</v>
+      </c>
+      <c r="F60" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G60" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H60" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>P-1060</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Lara Okada</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="D61" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E61" t="str">
+        <v>skeptical</v>
+      </c>
+      <c r="F61" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G61" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H61" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>P-1061</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Bruno Silva</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Lisbon</v>
+      </c>
+      <c r="D62" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E62" t="str">
+        <v>supportive</v>
+      </c>
+      <c r="F62" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G62" t="str">
+        <v>general</v>
+      </c>
+      <c r="H62" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>P-1062</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Nadia Keller</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Toronto</v>
+      </c>
+      <c r="D63" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E63" t="str">
+        <v>reserved</v>
+      </c>
+      <c r="F63" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G63" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H63" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>P-1063</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Elias Petrov</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Nairobi</v>
+      </c>
+      <c r="D64" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E64" t="str">
+        <v>playful</v>
+      </c>
+      <c r="F64" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G64" t="str">
+        <v>community</v>
+      </c>
+      <c r="H64" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>P-1064</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Tessa Voss</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Seoul</v>
+      </c>
+      <c r="D65" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E65" t="str">
+        <v>curious</v>
+      </c>
+      <c r="F65" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G65" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H65" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>P-1065</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Omar Adeyemi</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Mexico City</v>
+      </c>
+      <c r="D66" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E66" t="str">
+        <v>practical</v>
+      </c>
+      <c r="F66" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G66" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H66" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>P-1066</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Vera Berg</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Berlin</v>
+      </c>
+      <c r="D67" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E67" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F67" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G67" t="str">
+        <v>general</v>
+      </c>
+      <c r="H67" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>P-1067</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Jamal Ibrahim</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="D68" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E68" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F68" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G68" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H68" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>P-1068</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Cora Lind</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Vienna</v>
+      </c>
+      <c r="D69" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E69" t="str">
+        <v>enthusiastic</v>
+      </c>
+      <c r="F69" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G69" t="str">
+        <v>community</v>
+      </c>
+      <c r="H69" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>P-1069</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Rafa Mwangi</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Lagos</v>
+      </c>
+      <c r="D70" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E70" t="str">
+        <v>skeptical</v>
+      </c>
+      <c r="F70" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G70" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H70" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>P-1070</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Mina Park</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Milan</v>
+      </c>
+      <c r="D71" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E71" t="str">
+        <v>supportive</v>
+      </c>
+      <c r="F71" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G71" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H71" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>P-1071</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Nia Hale</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Austin</v>
+      </c>
+      <c r="D72" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E72" t="str">
+        <v>reserved</v>
+      </c>
+      <c r="F72" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G72" t="str">
+        <v>general</v>
+      </c>
+      <c r="H72" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>P-1072</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Omar Duarte</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Singapore</v>
+      </c>
+      <c r="D73" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E73" t="str">
+        <v>playful</v>
+      </c>
+      <c r="F73" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G73" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H73" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>P-1073</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Sable Patel</v>
+      </c>
+      <c r="C74" t="str">
+        <v>São Paulo</v>
+      </c>
+      <c r="D74" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E74" t="str">
+        <v>curious</v>
+      </c>
+      <c r="F74" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G74" t="str">
+        <v>community</v>
+      </c>
+      <c r="H74" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>P-1074</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Jun Bauer</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Osaka</v>
+      </c>
+      <c r="D75" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E75" t="str">
+        <v>practical</v>
+      </c>
+      <c r="F75" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G75" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H75" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>P-1075</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Mira Romano</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Cairo</v>
+      </c>
+      <c r="D76" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E76" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F76" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G76" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H76" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>P-1076</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Theo Brandt</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Stockholm</v>
+      </c>
+      <c r="D77" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E77" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F77" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G77" t="str">
+        <v>general</v>
+      </c>
+      <c r="H77" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>P-1077</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Asha Alvarez</v>
+      </c>
+      <c r="C78" t="str">
+        <v>London</v>
+      </c>
+      <c r="D78" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E78" t="str">
+        <v>enthusiastic</v>
+      </c>
+      <c r="F78" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G78" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H78" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>P-1078</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Lina Cho</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Accra</v>
+      </c>
+      <c r="D79" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E79" t="str">
+        <v>skeptical</v>
+      </c>
+      <c r="F79" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G79" t="str">
+        <v>community</v>
+      </c>
+      <c r="H79" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>P-1079</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Chris Rahman</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Chicago</v>
+      </c>
+      <c r="D80" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E80" t="str">
+        <v>supportive</v>
+      </c>
+      <c r="F80" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G80" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H80" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>P-1080</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Elena Nguyen</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="D81" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E81" t="str">
+        <v>reserved</v>
+      </c>
+      <c r="F81" t="str">
+        <v>concise</v>
+      </c>
+      <c r="G81" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H81" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>P-1081</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Quinn Calder</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Lisbon</v>
+      </c>
+      <c r="D82" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E82" t="str">
+        <v>playful</v>
+      </c>
+      <c r="F82" t="str">
+        <v>conversational</v>
+      </c>
+      <c r="G82" t="str">
+        <v>general</v>
+      </c>
+      <c r="H82" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>P-1082</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Priya Hock</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Toronto</v>
+      </c>
+      <c r="D83" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E83" t="str">
+        <v>curious</v>
+      </c>
+      <c r="F83" t="str">
+        <v>plain-language</v>
+      </c>
+      <c r="G83" t="str">
+        <v>procedural</v>
+      </c>
+      <c r="H83" t="str">
+        <v>low</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>P-1083</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Mateo Diallo</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Nairobi</v>
+      </c>
+      <c r="D84" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E84" t="str">
+        <v>practical</v>
+      </c>
+      <c r="F84" t="str">
+        <v>warm</v>
+      </c>
+      <c r="G84" t="str">
+        <v>community</v>
+      </c>
+      <c r="H84" t="str">
+        <v>moderate</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>P-1084</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Hana Novak</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Seoul</v>
+      </c>
+      <c r="D85" t="str">
+        <v>experienced</v>
+      </c>
+      <c r="E85" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="F85" t="str">
+        <v>precise</v>
+      </c>
+      <c r="G85" t="str">
+        <v>onboarding</v>
+      </c>
+      <c r="H85" t="str">
+        <v>high</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>P-1085</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Ibrahim Okafor</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Mexico City</v>
+      </c>
+      <c r="D86" t="str">
+        <v>beginner</v>
+      </c>
+      <c r="E86" t="str">
+        <v>calm</v>
+      </c>
+      <c r="F86" t="str">
+        <v>casual</v>
+      </c>
+      <c r="G86" t="str">
+        <v>faq</v>
+      </c>
+      <c r="H86" t="str">
         <v>low</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H86"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>